<commit_message>
## feat: implement location-based attendance tracking with time-limited QR sessions
</commit_message>
<xml_diff>
--- a/Attendance_Sheet.xlsx
+++ b/Attendance_Sheet.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,6 +435,31 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>18:08:13</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>25102A2006</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Present</t>
         </is>
       </c>
     </row>

</xml_diff>